<commit_message>
Test doc updated to include errors faced in deployment
</commit_message>
<xml_diff>
--- a/Documentation/SRS_HVPSU_Test_Results.xlsx
+++ b/Documentation/SRS_HVPSU_Test_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\home\jek48386\repos\SRS300\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2985331-0F0B-472F-AA27-ABBDDF0D4B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{442D95D0-0ED6-48A2-B7EC-ED21C98754DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1875" windowWidth="29040" windowHeight="15720" xr2:uid="{ABB50434-DF5E-4618-8107-94BD17379F73}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="223">
   <si>
     <t>Test</t>
   </si>
@@ -881,6 +881,14 @@
   </si>
   <si>
     <t>Deploy a second instance of the IOC</t>
+  </si>
+  <si>
+    <t>Errors when trying to deploy, did 
+not deploy.</t>
+  </si>
+  <si>
+    <t>Prefix contained a colon which
+ caused an error so it was removed and put into the PV name instead, Prefix was in two parts "$(P)$(R)" which caused some issues so it was changed to "$(DEVICE)"</t>
   </si>
 </sst>
 </file>
@@ -1665,7 +1673,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="227">
+  <cellXfs count="231">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1980,288 +1988,300 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2271,8 +2291,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFFFCC"/>
       <color rgb="FFEDFDCF"/>
-      <color rgb="FFFFFFCC"/>
       <color rgb="FFF9FEE2"/>
       <color rgb="FFF6FECE"/>
       <color rgb="FFDDFFFF"/>
@@ -2609,7 +2629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A62839A-462D-4B14-AC2D-C7655127CCDA}">
-  <dimension ref="A1:M119"/>
+  <dimension ref="A1:M120"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.28515625" style="1" customWidth="1"/>
@@ -2626,34 +2646,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="217" t="s">
         <v>211</v>
       </c>
-      <c r="B1" s="128"/>
+      <c r="B1" s="218"/>
       <c r="C1" s="122"/>
       <c r="D1" s="123"/>
       <c r="E1" s="121"/>
       <c r="F1" s="121"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="129" t="s">
+      <c r="A2" s="219" t="s">
         <v>210</v>
       </c>
-      <c r="B2" s="130"/>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="131"/>
+      <c r="B2" s="220"/>
+      <c r="C2" s="220"/>
+      <c r="D2" s="220"/>
+      <c r="E2" s="221"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="132" t="s">
+      <c r="A3" s="215" t="s">
         <v>212</v>
       </c>
-      <c r="B3" s="133"/>
-      <c r="C3" s="133"/>
-      <c r="D3" s="133"/>
-      <c r="E3" s="133"/>
+      <c r="B3" s="222"/>
+      <c r="C3" s="222"/>
+      <c r="D3" s="222"/>
+      <c r="E3" s="222"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
@@ -2666,10 +2686,10 @@
     </row>
     <row r="5" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="6" spans="1:13" s="4" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="163" t="s">
+      <c r="B6" s="202" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="164"/>
+      <c r="C6" s="203"/>
       <c r="D6" s="24" t="s">
         <v>206</v>
       </c>
@@ -2688,21 +2708,21 @@
       <c r="I6" s="86" t="s">
         <v>132</v>
       </c>
-      <c r="K6" s="155" t="s">
+      <c r="K6" s="201" t="s">
         <v>147</v>
       </c>
-      <c r="L6" s="155"/>
+      <c r="L6" s="201"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="165" t="s">
+      <c r="B7" s="204" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="166"/>
-      <c r="D7" s="166"/>
-      <c r="E7" s="166"/>
-      <c r="F7" s="166"/>
-      <c r="G7" s="166"/>
-      <c r="H7" s="166"/>
+      <c r="C7" s="205"/>
+      <c r="D7" s="205"/>
+      <c r="E7" s="205"/>
+      <c r="F7" s="205"/>
+      <c r="G7" s="205"/>
+      <c r="H7" s="205"/>
       <c r="I7" s="91"/>
       <c r="K7" s="13"/>
       <c r="L7" s="3" t="s">
@@ -2728,24 +2748,24 @@
       </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="156" t="s">
+      <c r="B9" s="180" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="145" t="s">
+      <c r="C9" s="191" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="159"/>
-      <c r="E9" s="162" t="s">
+      <c r="D9" s="197"/>
+      <c r="E9" s="198" t="s">
         <v>69</v>
       </c>
-      <c r="F9" s="173" t="s">
-        <v>130</v>
-      </c>
-      <c r="G9" s="167">
+      <c r="F9" s="212" t="s">
+        <v>130</v>
+      </c>
+      <c r="G9" s="206">
         <v>45992</v>
       </c>
-      <c r="H9" s="170"/>
-      <c r="I9" s="148" t="s">
+      <c r="H9" s="209"/>
+      <c r="I9" s="166" t="s">
         <v>131</v>
       </c>
       <c r="K9" s="15"/>
@@ -2754,38 +2774,38 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="157"/>
-      <c r="C10" s="146"/>
-      <c r="D10" s="160"/>
-      <c r="E10" s="141"/>
-      <c r="F10" s="174"/>
-      <c r="G10" s="168"/>
-      <c r="H10" s="171"/>
-      <c r="I10" s="136"/>
+      <c r="B10" s="165"/>
+      <c r="C10" s="174"/>
+      <c r="D10" s="182"/>
+      <c r="E10" s="176"/>
+      <c r="F10" s="213"/>
+      <c r="G10" s="207"/>
+      <c r="H10" s="210"/>
+      <c r="I10" s="170"/>
       <c r="K10" s="19"/>
       <c r="L10" s="2" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="157"/>
-      <c r="C11" s="146"/>
-      <c r="D11" s="160"/>
-      <c r="E11" s="141"/>
-      <c r="F11" s="174"/>
-      <c r="G11" s="168"/>
-      <c r="H11" s="171"/>
-      <c r="I11" s="136"/>
+      <c r="B11" s="165"/>
+      <c r="C11" s="174"/>
+      <c r="D11" s="182"/>
+      <c r="E11" s="176"/>
+      <c r="F11" s="213"/>
+      <c r="G11" s="207"/>
+      <c r="H11" s="210"/>
+      <c r="I11" s="170"/>
     </row>
     <row r="12" spans="1:13" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="158"/>
-      <c r="C12" s="147"/>
-      <c r="D12" s="161"/>
-      <c r="E12" s="144"/>
-      <c r="F12" s="175"/>
-      <c r="G12" s="169"/>
-      <c r="H12" s="172"/>
-      <c r="I12" s="137"/>
+      <c r="B12" s="153"/>
+      <c r="C12" s="155"/>
+      <c r="D12" s="157"/>
+      <c r="E12" s="177"/>
+      <c r="F12" s="214"/>
+      <c r="G12" s="208"/>
+      <c r="H12" s="211"/>
+      <c r="I12" s="167"/>
       <c r="M12" s="12"/>
     </row>
     <row r="13" spans="1:13" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2833,13 +2853,13 @@
       </c>
     </row>
     <row r="15" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="176" t="s">
+      <c r="B15" s="152" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="134" t="s">
+      <c r="C15" s="185" t="s">
         <v>24</v>
       </c>
-      <c r="D15" s="134" t="s">
+      <c r="D15" s="185" t="s">
         <v>73</v>
       </c>
       <c r="E15" s="37" t="s">
@@ -2852,14 +2872,14 @@
         <v>45989</v>
       </c>
       <c r="H15" s="93"/>
-      <c r="I15" s="148" t="s">
+      <c r="I15" s="166" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="158"/>
-      <c r="C16" s="135"/>
-      <c r="D16" s="135"/>
+      <c r="B16" s="153"/>
+      <c r="C16" s="187"/>
+      <c r="D16" s="187"/>
       <c r="E16" s="31" t="s">
         <v>74</v>
       </c>
@@ -2870,7 +2890,7 @@
         <v>45989</v>
       </c>
       <c r="H16" s="94"/>
-      <c r="I16" s="137"/>
+      <c r="I16" s="167"/>
     </row>
     <row r="17" spans="2:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="63" t="s">
@@ -2911,13 +2931,13 @@
       <c r="I18" s="85"/>
     </row>
     <row r="19" spans="2:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="156" t="s">
+      <c r="B19" s="180" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="132" t="s">
+      <c r="C19" s="215" t="s">
         <v>79</v>
       </c>
-      <c r="D19" s="145"/>
+      <c r="D19" s="191"/>
       <c r="E19" s="22" t="s">
         <v>77</v>
       </c>
@@ -2928,14 +2948,14 @@
         <v>45992</v>
       </c>
       <c r="H19" s="96"/>
-      <c r="I19" s="150" t="s">
+      <c r="I19" s="168" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="157"/>
-      <c r="C20" s="177"/>
-      <c r="D20" s="146"/>
+      <c r="B20" s="165"/>
+      <c r="C20" s="186"/>
+      <c r="D20" s="174"/>
       <c r="E20" s="5" t="s">
         <v>78</v>
       </c>
@@ -2946,12 +2966,12 @@
         <v>45992</v>
       </c>
       <c r="H20" s="74"/>
-      <c r="I20" s="136"/>
+      <c r="I20" s="170"/>
     </row>
     <row r="21" spans="2:9" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="158"/>
-      <c r="C21" s="135"/>
-      <c r="D21" s="147"/>
+      <c r="B21" s="153"/>
+      <c r="C21" s="187"/>
+      <c r="D21" s="155"/>
       <c r="E21" s="31" t="s">
         <v>80</v>
       </c>
@@ -2962,16 +2982,16 @@
         <v>45992</v>
       </c>
       <c r="H21" s="94"/>
-      <c r="I21" s="137"/>
+      <c r="I21" s="167"/>
     </row>
     <row r="22" spans="2:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="B22" s="176" t="s">
+      <c r="B22" s="152" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="134" t="s">
+      <c r="C22" s="185" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="134"/>
+      <c r="D22" s="185"/>
       <c r="E22" s="30" t="s">
         <v>81</v>
       </c>
@@ -2982,14 +3002,14 @@
         <v>45992</v>
       </c>
       <c r="H22" s="93"/>
-      <c r="I22" s="148" t="s">
+      <c r="I22" s="166" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="23" spans="2:9" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="158"/>
-      <c r="C23" s="135"/>
-      <c r="D23" s="135"/>
+      <c r="B23" s="153"/>
+      <c r="C23" s="187"/>
+      <c r="D23" s="187"/>
       <c r="E23" s="31" t="s">
         <v>82</v>
       </c>
@@ -3000,16 +3020,16 @@
         <v>45992</v>
       </c>
       <c r="H23" s="94"/>
-      <c r="I23" s="137"/>
+      <c r="I23" s="167"/>
     </row>
     <row r="24" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B24" s="176" t="s">
+      <c r="B24" s="152" t="s">
         <v>54</v>
       </c>
-      <c r="C24" s="134" t="s">
+      <c r="C24" s="185" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="134"/>
+      <c r="D24" s="185"/>
       <c r="E24" s="30" t="s">
         <v>83</v>
       </c>
@@ -3025,10 +3045,10 @@
       </c>
     </row>
     <row r="25" spans="2:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B25" s="157"/>
-      <c r="C25" s="177"/>
-      <c r="D25" s="177"/>
-      <c r="E25" s="141" t="s">
+      <c r="B25" s="165"/>
+      <c r="C25" s="186"/>
+      <c r="D25" s="186"/>
+      <c r="E25" s="176" t="s">
         <v>84</v>
       </c>
       <c r="F25" s="17" t="s">
@@ -3040,15 +3060,15 @@
       <c r="H25" s="97" t="s">
         <v>187</v>
       </c>
-      <c r="I25" s="136" t="s">
+      <c r="I25" s="170" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="26" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="158"/>
-      <c r="C26" s="135"/>
-      <c r="D26" s="135"/>
-      <c r="E26" s="144"/>
+      <c r="B26" s="153"/>
+      <c r="C26" s="187"/>
+      <c r="D26" s="187"/>
+      <c r="E26" s="177"/>
       <c r="F26" s="39" t="s">
         <v>130</v>
       </c>
@@ -3056,16 +3076,16 @@
         <v>45989</v>
       </c>
       <c r="H26" s="98"/>
-      <c r="I26" s="137"/>
+      <c r="I26" s="167"/>
     </row>
     <row r="27" spans="2:9" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="176" t="s">
+      <c r="B27" s="152" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="134" t="s">
+      <c r="C27" s="185" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="134"/>
+      <c r="D27" s="185"/>
       <c r="E27" s="30" t="s">
         <v>85</v>
       </c>
@@ -3081,10 +3101,10 @@
       </c>
     </row>
     <row r="28" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="157"/>
-      <c r="C28" s="177"/>
-      <c r="D28" s="177"/>
-      <c r="E28" s="141" t="s">
+      <c r="B28" s="165"/>
+      <c r="C28" s="186"/>
+      <c r="D28" s="186"/>
+      <c r="E28" s="176" t="s">
         <v>86</v>
       </c>
       <c r="F28" s="17" t="s">
@@ -3096,15 +3116,15 @@
       <c r="H28" s="97" t="s">
         <v>187</v>
       </c>
-      <c r="I28" s="136" t="s">
+      <c r="I28" s="170" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="29" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="158"/>
-      <c r="C29" s="135"/>
-      <c r="D29" s="135"/>
-      <c r="E29" s="144"/>
+      <c r="B29" s="153"/>
+      <c r="C29" s="187"/>
+      <c r="D29" s="187"/>
+      <c r="E29" s="177"/>
       <c r="F29" s="41" t="s">
         <v>130</v>
       </c>
@@ -3112,7 +3132,7 @@
         <v>45988</v>
       </c>
       <c r="H29" s="99"/>
-      <c r="I29" s="137"/>
+      <c r="I29" s="167"/>
     </row>
     <row r="30" spans="2:9" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="32" t="s">
@@ -3173,13 +3193,13 @@
       </c>
     </row>
     <row r="33" spans="2:12" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="156">
+      <c r="B33" s="180">
         <v>2.2000000000000002</v>
       </c>
-      <c r="C33" s="145" t="s">
+      <c r="C33" s="191" t="s">
         <v>91</v>
       </c>
-      <c r="D33" s="145" t="s">
+      <c r="D33" s="191" t="s">
         <v>94</v>
       </c>
       <c r="E33" s="22" t="s">
@@ -3197,10 +3217,10 @@
       </c>
     </row>
     <row r="34" spans="2:12" ht="60" x14ac:dyDescent="0.25">
-      <c r="B34" s="157"/>
-      <c r="C34" s="146"/>
-      <c r="D34" s="146"/>
-      <c r="E34" s="141" t="s">
+      <c r="B34" s="165"/>
+      <c r="C34" s="174"/>
+      <c r="D34" s="174"/>
+      <c r="E34" s="176" t="s">
         <v>93</v>
       </c>
       <c r="F34" s="16" t="s">
@@ -3212,15 +3232,15 @@
       <c r="H34" s="100" t="s">
         <v>190</v>
       </c>
-      <c r="I34" s="148" t="s">
+      <c r="I34" s="166" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="35" spans="2:12" ht="60" x14ac:dyDescent="0.25">
-      <c r="B35" s="157"/>
-      <c r="C35" s="146"/>
-      <c r="D35" s="146"/>
-      <c r="E35" s="141"/>
+      <c r="B35" s="165"/>
+      <c r="C35" s="174"/>
+      <c r="D35" s="174"/>
+      <c r="E35" s="176"/>
       <c r="F35" s="16" t="s">
         <v>191</v>
       </c>
@@ -3230,13 +3250,13 @@
       <c r="H35" s="97" t="s">
         <v>192</v>
       </c>
-      <c r="I35" s="136"/>
+      <c r="I35" s="170"/>
     </row>
     <row r="36" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="186"/>
-      <c r="C36" s="154"/>
-      <c r="D36" s="154"/>
-      <c r="E36" s="183"/>
+      <c r="B36" s="181"/>
+      <c r="C36" s="184"/>
+      <c r="D36" s="184"/>
+      <c r="E36" s="192"/>
       <c r="F36" s="43" t="s">
         <v>130</v>
       </c>
@@ -3244,16 +3264,16 @@
         <v>45989</v>
       </c>
       <c r="H36" s="101"/>
-      <c r="I36" s="137"/>
+      <c r="I36" s="167"/>
     </row>
     <row r="37" spans="2:12" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="176">
+      <c r="B37" s="152">
         <v>2.2999999999999998</v>
       </c>
-      <c r="C37" s="180" t="s">
+      <c r="C37" s="154" t="s">
         <v>30</v>
       </c>
-      <c r="D37" s="180"/>
+      <c r="D37" s="154"/>
       <c r="E37" s="30" t="s">
         <v>95</v>
       </c>
@@ -3271,10 +3291,10 @@
       </c>
     </row>
     <row r="38" spans="2:12" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="157"/>
-      <c r="C38" s="146"/>
-      <c r="D38" s="146"/>
-      <c r="E38" s="141" t="s">
+      <c r="B38" s="165"/>
+      <c r="C38" s="174"/>
+      <c r="D38" s="174"/>
+      <c r="E38" s="176" t="s">
         <v>96</v>
       </c>
       <c r="F38" s="6" t="s">
@@ -3286,15 +3306,15 @@
       <c r="H38" s="97" t="s">
         <v>129</v>
       </c>
-      <c r="I38" s="150" t="s">
+      <c r="I38" s="168" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="39" spans="2:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="158"/>
-      <c r="C39" s="147"/>
-      <c r="D39" s="147"/>
-      <c r="E39" s="144"/>
+      <c r="B39" s="153"/>
+      <c r="C39" s="155"/>
+      <c r="D39" s="155"/>
+      <c r="E39" s="177"/>
       <c r="F39" s="31" t="s">
         <v>130</v>
       </c>
@@ -3302,16 +3322,16 @@
         <v>45981</v>
       </c>
       <c r="H39" s="94"/>
-      <c r="I39" s="137"/>
+      <c r="I39" s="167"/>
     </row>
     <row r="40" spans="2:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="B40" s="156">
+      <c r="B40" s="180">
         <v>2.4</v>
       </c>
-      <c r="C40" s="132" t="s">
+      <c r="C40" s="215" t="s">
         <v>23</v>
       </c>
-      <c r="D40" s="145"/>
+      <c r="D40" s="191"/>
       <c r="E40" s="22" t="s">
         <v>97</v>
       </c>
@@ -3322,14 +3342,14 @@
         <v>45992</v>
       </c>
       <c r="H40" s="96"/>
-      <c r="I40" s="150" t="s">
+      <c r="I40" s="168" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="41" spans="2:12" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="186"/>
-      <c r="C41" s="178"/>
-      <c r="D41" s="154"/>
+      <c r="B41" s="181"/>
+      <c r="C41" s="216"/>
+      <c r="D41" s="184"/>
       <c r="E41" s="20" t="s">
         <v>98</v>
       </c>
@@ -3340,7 +3360,7 @@
         <v>45992</v>
       </c>
       <c r="H41" s="103"/>
-      <c r="I41" s="151"/>
+      <c r="I41" s="169"/>
     </row>
     <row r="42" spans="2:12" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="32">
@@ -3387,15 +3407,15 @@
       </c>
     </row>
     <row r="44" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="193" t="s">
+      <c r="B44" s="144" t="s">
         <v>60</v>
       </c>
-      <c r="C44" s="194"/>
-      <c r="D44" s="194"/>
-      <c r="E44" s="194"/>
-      <c r="F44" s="194"/>
-      <c r="G44" s="194"/>
-      <c r="H44" s="195"/>
+      <c r="C44" s="145"/>
+      <c r="D44" s="145"/>
+      <c r="E44" s="145"/>
+      <c r="F44" s="145"/>
+      <c r="G44" s="145"/>
+      <c r="H44" s="146"/>
       <c r="I44" s="58"/>
       <c r="L44" s="1"/>
     </row>
@@ -3432,7 +3452,7 @@
       <c r="E46" s="48" t="s">
         <v>102</v>
       </c>
-      <c r="F46" s="142" t="s">
+      <c r="F46" s="225" t="s">
         <v>185</v>
       </c>
       <c r="G46" s="51">
@@ -3454,7 +3474,7 @@
       <c r="E47" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="F47" s="143"/>
+      <c r="F47" s="226"/>
       <c r="G47" s="50">
         <v>45989</v>
       </c>
@@ -3486,15 +3506,15 @@
       </c>
     </row>
     <row r="49" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="199" t="s">
+      <c r="B49" s="147" t="s">
         <v>68</v>
       </c>
-      <c r="C49" s="200"/>
-      <c r="D49" s="200"/>
-      <c r="E49" s="200"/>
-      <c r="F49" s="200"/>
-      <c r="G49" s="200"/>
-      <c r="H49" s="201"/>
+      <c r="C49" s="148"/>
+      <c r="D49" s="148"/>
+      <c r="E49" s="148"/>
+      <c r="F49" s="148"/>
+      <c r="G49" s="148"/>
+      <c r="H49" s="149"/>
       <c r="I49" s="58"/>
     </row>
     <row r="50" spans="2:12" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3565,15 +3585,15 @@
       <c r="L52"/>
     </row>
     <row r="53" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B53" s="197" t="s">
+      <c r="B53" s="150" t="s">
         <v>67</v>
       </c>
-      <c r="C53" s="198"/>
-      <c r="D53" s="198"/>
-      <c r="E53" s="198"/>
-      <c r="F53" s="198"/>
-      <c r="G53" s="198"/>
-      <c r="H53" s="198"/>
+      <c r="C53" s="151"/>
+      <c r="D53" s="151"/>
+      <c r="E53" s="151"/>
+      <c r="F53" s="151"/>
+      <c r="G53" s="151"/>
+      <c r="H53" s="151"/>
       <c r="I53" s="58"/>
       <c r="L53" s="1"/>
     </row>
@@ -3666,15 +3686,15 @@
       </c>
     </row>
     <row r="58" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="124" t="s">
+      <c r="B58" s="171" t="s">
         <v>66</v>
       </c>
-      <c r="C58" s="125"/>
-      <c r="D58" s="125"/>
-      <c r="E58" s="125"/>
-      <c r="F58" s="125"/>
-      <c r="G58" s="125"/>
-      <c r="H58" s="125"/>
+      <c r="C58" s="172"/>
+      <c r="D58" s="172"/>
+      <c r="E58" s="172"/>
+      <c r="F58" s="172"/>
+      <c r="G58" s="172"/>
+      <c r="H58" s="172"/>
       <c r="I58" s="58"/>
     </row>
     <row r="59" spans="2:12" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3700,13 +3720,13 @@
       </c>
     </row>
     <row r="60" spans="2:12" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="176">
+      <c r="B60" s="152">
         <v>6.2</v>
       </c>
-      <c r="C60" s="180" t="s">
+      <c r="C60" s="154" t="s">
         <v>16</v>
       </c>
-      <c r="D60" s="180"/>
+      <c r="D60" s="154"/>
       <c r="E60" s="69" t="s">
         <v>153</v>
       </c>
@@ -3722,10 +3742,10 @@
       </c>
     </row>
     <row r="61" spans="2:12" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="157"/>
-      <c r="C61" s="146"/>
-      <c r="D61" s="146"/>
-      <c r="E61" s="141" t="s">
+      <c r="B61" s="165"/>
+      <c r="C61" s="174"/>
+      <c r="D61" s="174"/>
+      <c r="E61" s="176" t="s">
         <v>154</v>
       </c>
       <c r="F61" s="16" t="s">
@@ -3737,15 +3757,15 @@
       <c r="H61" s="100" t="s">
         <v>162</v>
       </c>
-      <c r="I61" s="148" t="s">
+      <c r="I61" s="166" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="62" spans="2:12" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="158"/>
-      <c r="C62" s="147"/>
-      <c r="D62" s="147"/>
-      <c r="E62" s="144"/>
+      <c r="B62" s="153"/>
+      <c r="C62" s="155"/>
+      <c r="D62" s="155"/>
+      <c r="E62" s="177"/>
       <c r="F62" s="41" t="s">
         <v>130</v>
       </c>
@@ -3753,7 +3773,7 @@
         <v>45985</v>
       </c>
       <c r="H62" s="99"/>
-      <c r="I62" s="137"/>
+      <c r="I62" s="167"/>
     </row>
     <row r="63" spans="2:12" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B63" s="18">
@@ -3778,28 +3798,28 @@
       </c>
     </row>
     <row r="64" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="191" t="s">
+      <c r="B64" s="163" t="s">
         <v>65</v>
       </c>
-      <c r="C64" s="192"/>
-      <c r="D64" s="192"/>
-      <c r="E64" s="192"/>
-      <c r="F64" s="192"/>
-      <c r="G64" s="192"/>
-      <c r="H64" s="192"/>
+      <c r="C64" s="164"/>
+      <c r="D64" s="164"/>
+      <c r="E64" s="164"/>
+      <c r="F64" s="164"/>
+      <c r="G64" s="164"/>
+      <c r="H64" s="164"/>
       <c r="I64" s="58"/>
     </row>
     <row r="65" spans="2:9" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="176">
+      <c r="B65" s="152">
         <v>7.1</v>
       </c>
-      <c r="C65" s="180" t="s">
+      <c r="C65" s="154" t="s">
         <v>163</v>
       </c>
-      <c r="D65" s="180" t="s">
+      <c r="D65" s="154" t="s">
         <v>164</v>
       </c>
-      <c r="E65" s="149" t="s">
+      <c r="E65" s="175" t="s">
         <v>170</v>
       </c>
       <c r="F65" s="30" t="s">
@@ -3808,46 +3828,46 @@
       <c r="G65" s="38">
         <v>45985</v>
       </c>
-      <c r="H65" s="139" t="s">
+      <c r="H65" s="223" t="s">
         <v>174</v>
       </c>
-      <c r="I65" s="148" t="s">
+      <c r="I65" s="166" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="66" spans="2:9" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="157"/>
-      <c r="C66" s="146"/>
-      <c r="D66" s="146"/>
-      <c r="E66" s="141"/>
+      <c r="B66" s="165"/>
+      <c r="C66" s="174"/>
+      <c r="D66" s="174"/>
+      <c r="E66" s="176"/>
       <c r="F66" s="6" t="s">
         <v>171</v>
       </c>
       <c r="G66" s="11">
         <v>45985</v>
       </c>
-      <c r="H66" s="140"/>
-      <c r="I66" s="136"/>
+      <c r="H66" s="224"/>
+      <c r="I66" s="170"/>
     </row>
     <row r="67" spans="2:9" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="157"/>
-      <c r="C67" s="146"/>
-      <c r="D67" s="146"/>
-      <c r="E67" s="141"/>
+      <c r="B67" s="165"/>
+      <c r="C67" s="174"/>
+      <c r="D67" s="174"/>
+      <c r="E67" s="176"/>
       <c r="F67" s="6" t="s">
         <v>173</v>
       </c>
       <c r="G67" s="11">
         <v>45985</v>
       </c>
-      <c r="H67" s="140"/>
-      <c r="I67" s="136"/>
+      <c r="H67" s="224"/>
+      <c r="I67" s="170"/>
     </row>
     <row r="68" spans="2:9" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="158"/>
-      <c r="C68" s="147"/>
-      <c r="D68" s="147"/>
-      <c r="E68" s="144"/>
+      <c r="B68" s="153"/>
+      <c r="C68" s="155"/>
+      <c r="D68" s="155"/>
+      <c r="E68" s="177"/>
       <c r="F68" s="41" t="s">
         <v>130</v>
       </c>
@@ -3855,16 +3875,16 @@
         <v>45995</v>
       </c>
       <c r="H68" s="94"/>
-      <c r="I68" s="137"/>
+      <c r="I68" s="167"/>
     </row>
     <row r="69" spans="2:9" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="156">
+      <c r="B69" s="180">
         <v>7.2</v>
       </c>
-      <c r="C69" s="145" t="s">
+      <c r="C69" s="191" t="s">
         <v>17</v>
       </c>
-      <c r="D69" s="145"/>
+      <c r="D69" s="191"/>
       <c r="E69" s="28" t="s">
         <v>112</v>
       </c>
@@ -3880,10 +3900,10 @@
       </c>
     </row>
     <row r="70" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="157"/>
-      <c r="C70" s="146"/>
-      <c r="D70" s="146"/>
-      <c r="E70" s="141" t="s">
+      <c r="B70" s="165"/>
+      <c r="C70" s="174"/>
+      <c r="D70" s="174"/>
+      <c r="E70" s="176" t="s">
         <v>177</v>
       </c>
       <c r="F70" s="16" t="s">
@@ -3895,15 +3915,15 @@
       <c r="H70" s="100" t="s">
         <v>175</v>
       </c>
-      <c r="I70" s="148" t="s">
+      <c r="I70" s="166" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="71" spans="2:9" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="157"/>
-      <c r="C71" s="146"/>
-      <c r="D71" s="146"/>
-      <c r="E71" s="141"/>
+      <c r="B71" s="165"/>
+      <c r="C71" s="174"/>
+      <c r="D71" s="174"/>
+      <c r="E71" s="176"/>
       <c r="F71" s="5" t="s">
         <v>130</v>
       </c>
@@ -3911,13 +3931,13 @@
         <v>45980</v>
       </c>
       <c r="H71" s="100"/>
-      <c r="I71" s="137"/>
+      <c r="I71" s="167"/>
     </row>
     <row r="72" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="157"/>
-      <c r="C72" s="146"/>
-      <c r="D72" s="146"/>
-      <c r="E72" s="141" t="s">
+      <c r="B72" s="165"/>
+      <c r="C72" s="174"/>
+      <c r="D72" s="174"/>
+      <c r="E72" s="176" t="s">
         <v>178</v>
       </c>
       <c r="F72" s="6" t="s">
@@ -3927,15 +3947,15 @@
       <c r="H72" s="100" t="s">
         <v>195</v>
       </c>
-      <c r="I72" s="150" t="s">
+      <c r="I72" s="168" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="73" spans="2:9" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="186"/>
-      <c r="C73" s="154"/>
-      <c r="D73" s="154"/>
-      <c r="E73" s="183"/>
+      <c r="B73" s="181"/>
+      <c r="C73" s="184"/>
+      <c r="D73" s="184"/>
+      <c r="E73" s="192"/>
       <c r="F73" s="20" t="s">
         <v>130</v>
       </c>
@@ -3943,19 +3963,19 @@
         <v>45992</v>
       </c>
       <c r="H73" s="101"/>
-      <c r="I73" s="151"/>
+      <c r="I73" s="169"/>
     </row>
     <row r="74" spans="2:9" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="176">
+      <c r="B74" s="152">
         <v>7.3</v>
       </c>
-      <c r="C74" s="180" t="s">
+      <c r="C74" s="154" t="s">
         <v>18</v>
       </c>
-      <c r="D74" s="134" t="s">
+      <c r="D74" s="185" t="s">
         <v>165</v>
       </c>
-      <c r="E74" s="196" t="s">
+      <c r="E74" s="178" t="s">
         <v>113</v>
       </c>
       <c r="F74" s="71" t="s">
@@ -3967,15 +3987,15 @@
       <c r="H74" s="107" t="s">
         <v>166</v>
       </c>
-      <c r="I74" s="148" t="s">
+      <c r="I74" s="166" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="75" spans="2:9" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="157"/>
-      <c r="C75" s="146"/>
-      <c r="D75" s="177"/>
-      <c r="E75" s="138"/>
+      <c r="B75" s="165"/>
+      <c r="C75" s="174"/>
+      <c r="D75" s="186"/>
+      <c r="E75" s="179"/>
       <c r="F75" s="9" t="s">
         <v>130</v>
       </c>
@@ -3983,13 +4003,13 @@
         <v>45933</v>
       </c>
       <c r="H75" s="100"/>
-      <c r="I75" s="151"/>
+      <c r="I75" s="169"/>
     </row>
     <row r="76" spans="2:9" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B76" s="157"/>
-      <c r="C76" s="146"/>
-      <c r="D76" s="177"/>
-      <c r="E76" s="138" t="s">
+      <c r="B76" s="165"/>
+      <c r="C76" s="174"/>
+      <c r="D76" s="186"/>
+      <c r="E76" s="179" t="s">
         <v>114</v>
       </c>
       <c r="F76" s="6" t="s">
@@ -4001,15 +4021,15 @@
       <c r="H76" s="100" t="s">
         <v>169</v>
       </c>
-      <c r="I76" s="148" t="s">
+      <c r="I76" s="166" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="77" spans="2:9" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="157"/>
-      <c r="C77" s="146"/>
-      <c r="D77" s="177"/>
-      <c r="E77" s="138"/>
+      <c r="B77" s="165"/>
+      <c r="C77" s="174"/>
+      <c r="D77" s="186"/>
+      <c r="E77" s="179"/>
       <c r="F77" s="8" t="s">
         <v>130</v>
       </c>
@@ -4017,12 +4037,12 @@
         <v>45967</v>
       </c>
       <c r="H77" s="74"/>
-      <c r="I77" s="137"/>
+      <c r="I77" s="167"/>
     </row>
     <row r="78" spans="2:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B78" s="158"/>
-      <c r="C78" s="147"/>
-      <c r="D78" s="135"/>
+      <c r="B78" s="153"/>
+      <c r="C78" s="155"/>
+      <c r="D78" s="187"/>
       <c r="E78" s="31" t="s">
         <v>115</v>
       </c>
@@ -4038,14 +4058,14 @@
       </c>
     </row>
     <row r="79" spans="2:9" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="176">
+      <c r="B79" s="152">
         <v>7.4</v>
       </c>
-      <c r="C79" s="180" t="s">
+      <c r="C79" s="154" t="s">
         <v>19</v>
       </c>
-      <c r="D79" s="180"/>
-      <c r="E79" s="149" t="s">
+      <c r="D79" s="154"/>
+      <c r="E79" s="175" t="s">
         <v>198</v>
       </c>
       <c r="F79" s="71" t="s">
@@ -4057,15 +4077,15 @@
       <c r="H79" s="102" t="s">
         <v>158</v>
       </c>
-      <c r="I79" s="148" t="s">
+      <c r="I79" s="166" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="80" spans="2:9" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B80" s="157"/>
-      <c r="C80" s="146"/>
-      <c r="D80" s="146"/>
-      <c r="E80" s="141"/>
+      <c r="B80" s="165"/>
+      <c r="C80" s="174"/>
+      <c r="D80" s="174"/>
+      <c r="E80" s="176"/>
       <c r="F80" s="6" t="s">
         <v>160</v>
       </c>
@@ -4075,13 +4095,13 @@
       <c r="H80" s="108" t="s">
         <v>161</v>
       </c>
-      <c r="I80" s="136"/>
+      <c r="I80" s="170"/>
     </row>
     <row r="81" spans="2:9" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="157"/>
-      <c r="C81" s="146"/>
-      <c r="D81" s="146"/>
-      <c r="E81" s="141"/>
+      <c r="B81" s="165"/>
+      <c r="C81" s="174"/>
+      <c r="D81" s="174"/>
+      <c r="E81" s="176"/>
       <c r="F81" s="6" t="s">
         <v>199</v>
       </c>
@@ -4091,13 +4111,13 @@
       <c r="H81" s="108" t="s">
         <v>200</v>
       </c>
-      <c r="I81" s="136"/>
+      <c r="I81" s="170"/>
     </row>
     <row r="82" spans="2:9" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B82" s="157"/>
-      <c r="C82" s="146"/>
-      <c r="D82" s="146"/>
-      <c r="E82" s="141"/>
+      <c r="B82" s="165"/>
+      <c r="C82" s="174"/>
+      <c r="D82" s="174"/>
+      <c r="E82" s="176"/>
       <c r="F82" s="8" t="s">
         <v>130</v>
       </c>
@@ -4105,13 +4125,13 @@
         <v>45995</v>
       </c>
       <c r="H82" s="108"/>
-      <c r="I82" s="137"/>
+      <c r="I82" s="167"/>
     </row>
     <row r="83" spans="2:9" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B83" s="157"/>
-      <c r="C83" s="146"/>
-      <c r="D83" s="146"/>
-      <c r="E83" s="141" t="s">
+      <c r="B83" s="165"/>
+      <c r="C83" s="174"/>
+      <c r="D83" s="174"/>
+      <c r="E83" s="176" t="s">
         <v>157</v>
       </c>
       <c r="F83" s="6" t="s">
@@ -4123,15 +4143,15 @@
       <c r="H83" s="97" t="s">
         <v>156</v>
       </c>
-      <c r="I83" s="150" t="s">
+      <c r="I83" s="168" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="84" spans="2:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B84" s="158"/>
-      <c r="C84" s="147"/>
-      <c r="D84" s="147"/>
-      <c r="E84" s="144"/>
+      <c r="B84" s="153"/>
+      <c r="C84" s="155"/>
+      <c r="D84" s="155"/>
+      <c r="E84" s="177"/>
       <c r="F84" s="31" t="s">
         <v>130</v>
       </c>
@@ -4139,28 +4159,28 @@
         <v>45987</v>
       </c>
       <c r="H84" s="94"/>
-      <c r="I84" s="137"/>
+      <c r="I84" s="167"/>
     </row>
     <row r="85" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B85" s="193" t="s">
+      <c r="B85" s="144" t="s">
         <v>64</v>
       </c>
-      <c r="C85" s="194"/>
-      <c r="D85" s="194"/>
-      <c r="E85" s="194"/>
-      <c r="F85" s="194"/>
-      <c r="G85" s="194"/>
-      <c r="H85" s="195"/>
+      <c r="C85" s="145"/>
+      <c r="D85" s="145"/>
+      <c r="E85" s="145"/>
+      <c r="F85" s="145"/>
+      <c r="G85" s="145"/>
+      <c r="H85" s="146"/>
       <c r="I85" s="58"/>
     </row>
     <row r="86" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B86" s="176">
+      <c r="B86" s="152">
         <v>8.1</v>
       </c>
-      <c r="C86" s="180" t="s">
+      <c r="C86" s="154" t="s">
         <v>34</v>
       </c>
-      <c r="D86" s="179"/>
+      <c r="D86" s="156"/>
       <c r="E86" s="30" t="s">
         <v>179</v>
       </c>
@@ -4171,14 +4191,14 @@
         <v>45980</v>
       </c>
       <c r="H86" s="93"/>
-      <c r="I86" s="148" t="s">
+      <c r="I86" s="166" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="87" spans="2:9" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B87" s="157"/>
-      <c r="C87" s="146"/>
-      <c r="D87" s="160"/>
+      <c r="B87" s="165"/>
+      <c r="C87" s="174"/>
+      <c r="D87" s="182"/>
       <c r="E87" s="5" t="s">
         <v>180</v>
       </c>
@@ -4189,12 +4209,12 @@
         <v>45980</v>
       </c>
       <c r="H87" s="74"/>
-      <c r="I87" s="152"/>
+      <c r="I87" s="199"/>
     </row>
     <row r="88" spans="2:9" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B88" s="158"/>
-      <c r="C88" s="147"/>
-      <c r="D88" s="161"/>
+      <c r="B88" s="153"/>
+      <c r="C88" s="155"/>
+      <c r="D88" s="157"/>
       <c r="E88" s="31" t="s">
         <v>181</v>
       </c>
@@ -4205,16 +4225,16 @@
         <v>45980</v>
       </c>
       <c r="H88" s="94"/>
-      <c r="I88" s="153"/>
+      <c r="I88" s="200"/>
     </row>
     <row r="89" spans="2:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B89" s="176">
+      <c r="B89" s="152">
         <v>8.1999999999999993</v>
       </c>
-      <c r="C89" s="180" t="s">
+      <c r="C89" s="154" t="s">
         <v>33</v>
       </c>
-      <c r="D89" s="179"/>
+      <c r="D89" s="156"/>
       <c r="E89" s="30" t="s">
         <v>116</v>
       </c>
@@ -4230,9 +4250,9 @@
       </c>
     </row>
     <row r="90" spans="2:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B90" s="158"/>
-      <c r="C90" s="147"/>
-      <c r="D90" s="161"/>
+      <c r="B90" s="153"/>
+      <c r="C90" s="155"/>
+      <c r="D90" s="157"/>
       <c r="E90" s="31" t="s">
         <v>117</v>
       </c>
@@ -4292,13 +4312,13 @@
       </c>
     </row>
     <row r="93" spans="2:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B93" s="176">
+      <c r="B93" s="152">
         <v>8.5</v>
       </c>
-      <c r="C93" s="180" t="s">
+      <c r="C93" s="154" t="s">
         <v>36</v>
       </c>
-      <c r="D93" s="179"/>
+      <c r="D93" s="156"/>
       <c r="E93" s="30" t="s">
         <v>120</v>
       </c>
@@ -4314,9 +4334,9 @@
       </c>
     </row>
     <row r="94" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B94" s="157"/>
-      <c r="C94" s="146"/>
-      <c r="D94" s="160"/>
+      <c r="B94" s="165"/>
+      <c r="C94" s="174"/>
+      <c r="D94" s="182"/>
       <c r="E94" s="5" t="s">
         <v>121</v>
       </c>
@@ -4332,10 +4352,10 @@
       </c>
     </row>
     <row r="95" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B95" s="157"/>
-      <c r="C95" s="146"/>
-      <c r="D95" s="160"/>
-      <c r="E95" s="141" t="s">
+      <c r="B95" s="165"/>
+      <c r="C95" s="174"/>
+      <c r="D95" s="182"/>
+      <c r="E95" s="176" t="s">
         <v>122</v>
       </c>
       <c r="F95" s="17" t="s">
@@ -4347,15 +4367,15 @@
       <c r="H95" s="100" t="s">
         <v>184</v>
       </c>
-      <c r="I95" s="136" t="s">
+      <c r="I95" s="170" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="96" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B96" s="186"/>
-      <c r="C96" s="154"/>
-      <c r="D96" s="187"/>
-      <c r="E96" s="183"/>
+      <c r="B96" s="181"/>
+      <c r="C96" s="184"/>
+      <c r="D96" s="183"/>
+      <c r="E96" s="192"/>
       <c r="F96" s="20" t="s">
         <v>130</v>
       </c>
@@ -4363,41 +4383,41 @@
         <v>45980</v>
       </c>
       <c r="H96" s="103"/>
-      <c r="I96" s="151"/>
+      <c r="I96" s="169"/>
     </row>
     <row r="97" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B97" s="184" t="s">
+      <c r="B97" s="195" t="s">
         <v>63</v>
       </c>
-      <c r="C97" s="185"/>
-      <c r="D97" s="185"/>
-      <c r="E97" s="185"/>
-      <c r="F97" s="185"/>
-      <c r="G97" s="185"/>
-      <c r="H97" s="185"/>
+      <c r="C97" s="196"/>
+      <c r="D97" s="196"/>
+      <c r="E97" s="196"/>
+      <c r="F97" s="196"/>
+      <c r="G97" s="196"/>
+      <c r="H97" s="196"/>
       <c r="I97" s="73"/>
     </row>
     <row r="98" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B98" s="181" t="s">
+      <c r="B98" s="193" t="s">
         <v>151</v>
       </c>
-      <c r="C98" s="182"/>
-      <c r="D98" s="182"/>
-      <c r="E98" s="182"/>
-      <c r="F98" s="182"/>
-      <c r="G98" s="182"/>
+      <c r="C98" s="194"/>
+      <c r="D98" s="194"/>
+      <c r="E98" s="194"/>
+      <c r="F98" s="194"/>
+      <c r="G98" s="194"/>
       <c r="H98" s="77"/>
       <c r="I98" s="118"/>
     </row>
     <row r="99" spans="2:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B99" s="156">
+      <c r="B99" s="180">
         <v>9.1</v>
       </c>
-      <c r="C99" s="145" t="s">
+      <c r="C99" s="191" t="s">
         <v>37</v>
       </c>
-      <c r="D99" s="159"/>
-      <c r="E99" s="162" t="s">
+      <c r="D99" s="197"/>
+      <c r="E99" s="198" t="s">
         <v>124</v>
       </c>
       <c r="F99" s="75" t="s">
@@ -4409,15 +4429,15 @@
       <c r="H99" s="96" t="s">
         <v>141</v>
       </c>
-      <c r="I99" s="150" t="s">
+      <c r="I99" s="168" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="100" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B100" s="157"/>
-      <c r="C100" s="146"/>
-      <c r="D100" s="160"/>
-      <c r="E100" s="141"/>
+      <c r="B100" s="165"/>
+      <c r="C100" s="174"/>
+      <c r="D100" s="182"/>
+      <c r="E100" s="176"/>
       <c r="F100" s="8" t="s">
         <v>140</v>
       </c>
@@ -4425,13 +4445,13 @@
         <v>45985</v>
       </c>
       <c r="H100" s="74"/>
-      <c r="I100" s="136"/>
+      <c r="I100" s="170"/>
     </row>
     <row r="101" spans="2:9" ht="81.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B101" s="157"/>
-      <c r="C101" s="146"/>
-      <c r="D101" s="160"/>
-      <c r="E101" s="141" t="s">
+      <c r="B101" s="165"/>
+      <c r="C101" s="174"/>
+      <c r="D101" s="182"/>
+      <c r="E101" s="176" t="s">
         <v>125</v>
       </c>
       <c r="F101" s="6" t="s">
@@ -4443,15 +4463,15 @@
       <c r="H101" s="97" t="s">
         <v>139</v>
       </c>
-      <c r="I101" s="136" t="s">
+      <c r="I101" s="170" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="102" spans="2:9" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B102" s="158"/>
-      <c r="C102" s="147"/>
-      <c r="D102" s="161"/>
-      <c r="E102" s="144"/>
+      <c r="B102" s="153"/>
+      <c r="C102" s="155"/>
+      <c r="D102" s="157"/>
+      <c r="E102" s="177"/>
       <c r="F102" s="31" t="s">
         <v>138</v>
       </c>
@@ -4459,7 +4479,7 @@
         <v>45985</v>
       </c>
       <c r="H102" s="98"/>
-      <c r="I102" s="137"/>
+      <c r="I102" s="167"/>
     </row>
     <row r="103" spans="2:9" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B103" s="18">
@@ -4484,14 +4504,14 @@
       </c>
     </row>
     <row r="104" spans="2:9" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B104" s="176">
+      <c r="B104" s="152">
         <v>9.3000000000000007</v>
       </c>
-      <c r="C104" s="180" t="s">
+      <c r="C104" s="154" t="s">
         <v>39</v>
       </c>
-      <c r="D104" s="179"/>
-      <c r="E104" s="149" t="s">
+      <c r="D104" s="156"/>
+      <c r="E104" s="175" t="s">
         <v>142</v>
       </c>
       <c r="F104" s="71" t="s">
@@ -4503,67 +4523,67 @@
       <c r="H104" s="102" t="s">
         <v>144</v>
       </c>
-      <c r="I104" s="148" t="s">
+      <c r="I104" s="166" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="105" spans="2:9" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B105" s="186"/>
-      <c r="C105" s="154"/>
-      <c r="D105" s="187"/>
-      <c r="E105" s="183"/>
-      <c r="F105" s="206" t="s">
+      <c r="B105" s="181"/>
+      <c r="C105" s="184"/>
+      <c r="D105" s="183"/>
+      <c r="E105" s="192"/>
+      <c r="F105" s="125" t="s">
         <v>145</v>
       </c>
       <c r="G105" s="44">
         <v>45982</v>
       </c>
       <c r="H105" s="103"/>
-      <c r="I105" s="151"/>
+      <c r="I105" s="169"/>
     </row>
     <row r="106" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B106" s="176">
+      <c r="B106" s="152">
         <v>9.4</v>
       </c>
-      <c r="C106" s="180" t="s">
+      <c r="C106" s="154" t="s">
         <v>40</v>
       </c>
-      <c r="D106" s="179"/>
-      <c r="E106" s="210" t="s">
+      <c r="D106" s="156"/>
+      <c r="E106" s="158" t="s">
         <v>127</v>
       </c>
-      <c r="F106" s="211" t="s">
+      <c r="F106" s="127" t="s">
         <v>146</v>
       </c>
       <c r="G106" s="38">
         <v>45982</v>
       </c>
-      <c r="H106" s="215" t="s">
+      <c r="H106" s="161" t="s">
         <v>217</v>
       </c>
-      <c r="I106" s="217" t="s">
+      <c r="I106" s="133" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="107" spans="2:9" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B107" s="213"/>
-      <c r="C107" s="203"/>
-      <c r="D107" s="204"/>
-      <c r="E107" s="205"/>
-      <c r="F107" s="214" t="s">
+      <c r="B107" s="136"/>
+      <c r="C107" s="138"/>
+      <c r="D107" s="140"/>
+      <c r="E107" s="159"/>
+      <c r="F107" s="128" t="s">
         <v>218</v>
       </c>
       <c r="G107" s="57">
         <v>46030</v>
       </c>
-      <c r="H107" s="216"/>
-      <c r="I107" s="218"/>
+      <c r="H107" s="162"/>
+      <c r="I107" s="134"/>
     </row>
     <row r="108" spans="2:9" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B108" s="158"/>
-      <c r="C108" s="147"/>
-      <c r="D108" s="161"/>
-      <c r="E108" s="212"/>
+      <c r="B108" s="153"/>
+      <c r="C108" s="155"/>
+      <c r="D108" s="157"/>
+      <c r="E108" s="160"/>
       <c r="F108" s="72" t="s">
         <v>130</v>
       </c>
@@ -4571,19 +4591,19 @@
         <v>46031</v>
       </c>
       <c r="H108" s="94"/>
-      <c r="I108" s="219"/>
+      <c r="I108" s="135"/>
     </row>
     <row r="109" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B109" s="207" t="s">
+      <c r="B109" s="142" t="s">
         <v>62</v>
       </c>
-      <c r="C109" s="208"/>
-      <c r="D109" s="208"/>
-      <c r="E109" s="208"/>
-      <c r="F109" s="208"/>
-      <c r="G109" s="208"/>
-      <c r="H109" s="208"/>
-      <c r="I109" s="209"/>
+      <c r="C109" s="143"/>
+      <c r="D109" s="143"/>
+      <c r="E109" s="143"/>
+      <c r="F109" s="143"/>
+      <c r="G109" s="143"/>
+      <c r="H109" s="143"/>
+      <c r="I109" s="126"/>
     </row>
     <row r="110" spans="2:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B110" s="32">
@@ -4602,7 +4622,7 @@
       <c r="G110" s="36">
         <v>46009</v>
       </c>
-      <c r="H110" s="225"/>
+      <c r="H110" s="131"/>
       <c r="I110" s="113" t="s">
         <v>131</v>
       </c>
@@ -4624,7 +4644,7 @@
       <c r="G111" s="36">
         <v>46009</v>
       </c>
-      <c r="H111" s="225"/>
+      <c r="H111" s="131"/>
       <c r="I111" s="112" t="s">
         <v>131</v>
       </c>
@@ -4636,28 +4656,28 @@
       <c r="C112" s="54" t="s">
         <v>43</v>
       </c>
-      <c r="D112" s="202" t="s">
+      <c r="D112" s="124" t="s">
         <v>215</v>
       </c>
-      <c r="E112" s="202" t="s">
+      <c r="E112" s="124" t="s">
         <v>216</v>
       </c>
-      <c r="F112" s="224"/>
-      <c r="G112" s="226"/>
+      <c r="F112" s="130"/>
+      <c r="G112" s="132"/>
       <c r="H112" s="106"/>
-      <c r="I112" s="220"/>
+      <c r="I112" s="129"/>
     </row>
     <row r="113" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B113" s="124" t="s">
+      <c r="B113" s="171" t="s">
         <v>61</v>
       </c>
-      <c r="C113" s="125"/>
-      <c r="D113" s="125"/>
-      <c r="E113" s="125"/>
-      <c r="F113" s="125"/>
-      <c r="G113" s="125"/>
-      <c r="H113" s="125"/>
-      <c r="I113" s="126"/>
+      <c r="C113" s="172"/>
+      <c r="D113" s="172"/>
+      <c r="E113" s="172"/>
+      <c r="F113" s="172"/>
+      <c r="G113" s="172"/>
+      <c r="H113" s="172"/>
+      <c r="I113" s="173"/>
     </row>
     <row r="114" spans="2:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B114" s="32">
@@ -4726,76 +4746,156 @@
       </c>
     </row>
     <row r="117" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B117" s="124" t="s">
+      <c r="B117" s="171" t="s">
         <v>208</v>
       </c>
-      <c r="C117" s="125"/>
-      <c r="D117" s="125"/>
-      <c r="E117" s="125"/>
-      <c r="F117" s="125"/>
-      <c r="G117" s="125"/>
-      <c r="H117" s="125"/>
-      <c r="I117" s="126"/>
-    </row>
-    <row r="118" spans="2:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B118" s="213">
+      <c r="C117" s="172"/>
+      <c r="D117" s="172"/>
+      <c r="E117" s="172"/>
+      <c r="F117" s="172"/>
+      <c r="G117" s="172"/>
+      <c r="H117" s="172"/>
+      <c r="I117" s="173"/>
+    </row>
+    <row r="118" spans="2:9" ht="109.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B118" s="136">
         <v>12.1</v>
       </c>
-      <c r="C118" s="203" t="s">
+      <c r="C118" s="138" t="s">
         <v>209</v>
       </c>
-      <c r="D118" s="204"/>
-      <c r="E118" s="22" t="s">
+      <c r="D118" s="140"/>
+      <c r="E118" s="227" t="s">
         <v>219</v>
       </c>
-      <c r="F118" s="42" t="s">
-        <v>130</v>
+      <c r="F118" s="229" t="s">
+        <v>221</v>
       </c>
       <c r="G118" s="29">
         <v>46028</v>
       </c>
-      <c r="H118" s="96"/>
+      <c r="H118" s="230" t="s">
+        <v>222</v>
+      </c>
       <c r="I118" s="112" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="119" spans="2:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B119" s="221"/>
-      <c r="C119" s="222"/>
-      <c r="D119" s="223"/>
-      <c r="E119" s="68" t="s">
+    <row r="119" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B119" s="136"/>
+      <c r="C119" s="138"/>
+      <c r="D119" s="140"/>
+      <c r="E119" s="228"/>
+      <c r="F119" s="42" t="s">
+        <v>130</v>
+      </c>
+      <c r="G119" s="29">
+        <v>46028</v>
+      </c>
+      <c r="H119" s="74"/>
+      <c r="I119" s="112"/>
+    </row>
+    <row r="120" spans="2:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B120" s="137"/>
+      <c r="C120" s="139"/>
+      <c r="D120" s="141"/>
+      <c r="E120" s="68" t="s">
         <v>220</v>
       </c>
-      <c r="F119" s="53" t="s">
-        <v>130</v>
-      </c>
-      <c r="G119" s="62">
+      <c r="F120" s="53" t="s">
+        <v>130</v>
+      </c>
+      <c r="G120" s="62">
         <v>46028</v>
       </c>
-      <c r="H119" s="105"/>
-      <c r="I119" s="112" t="s">
+      <c r="H120" s="105"/>
+      <c r="I120" s="112" t="s">
         <v>131</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="128">
-    <mergeCell ref="I106:I108"/>
-    <mergeCell ref="B118:B119"/>
-    <mergeCell ref="C118:C119"/>
-    <mergeCell ref="D118:D119"/>
-    <mergeCell ref="B109:H109"/>
-    <mergeCell ref="B44:H44"/>
-    <mergeCell ref="B49:H49"/>
-    <mergeCell ref="B53:H53"/>
-    <mergeCell ref="B106:B108"/>
-    <mergeCell ref="C106:C108"/>
-    <mergeCell ref="D106:D108"/>
-    <mergeCell ref="E106:E108"/>
-    <mergeCell ref="H106:H107"/>
-    <mergeCell ref="B64:H64"/>
-    <mergeCell ref="B85:H85"/>
-    <mergeCell ref="B74:B78"/>
-    <mergeCell ref="B79:B84"/>
+  <mergeCells count="129">
+    <mergeCell ref="E118:E119"/>
+    <mergeCell ref="B117:I117"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="I38:I39"/>
+    <mergeCell ref="E76:E77"/>
+    <mergeCell ref="H65:H67"/>
+    <mergeCell ref="E70:E71"/>
+    <mergeCell ref="F46:F47"/>
+    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="D19:D21"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="I65:I68"/>
+    <mergeCell ref="E79:E82"/>
+    <mergeCell ref="I79:I82"/>
+    <mergeCell ref="I19:I21"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="I28:I29"/>
+    <mergeCell ref="I34:I36"/>
+    <mergeCell ref="I70:I71"/>
+    <mergeCell ref="I72:I73"/>
+    <mergeCell ref="I74:I75"/>
+    <mergeCell ref="I86:I88"/>
+    <mergeCell ref="D69:D73"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="B9:B12"/>
+    <mergeCell ref="C9:C12"/>
+    <mergeCell ref="D9:D12"/>
+    <mergeCell ref="E9:E12"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="G9:G12"/>
+    <mergeCell ref="H9:H12"/>
+    <mergeCell ref="F9:F12"/>
+    <mergeCell ref="I9:I12"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="B89:B90"/>
+    <mergeCell ref="B93:B96"/>
+    <mergeCell ref="I104:I105"/>
+    <mergeCell ref="B99:B102"/>
+    <mergeCell ref="C99:C102"/>
+    <mergeCell ref="D99:D102"/>
+    <mergeCell ref="E101:E102"/>
+    <mergeCell ref="E99:E100"/>
+    <mergeCell ref="I99:I100"/>
+    <mergeCell ref="I101:I102"/>
+    <mergeCell ref="D104:D105"/>
+    <mergeCell ref="C104:C105"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="C27:C29"/>
+    <mergeCell ref="D27:D29"/>
+    <mergeCell ref="B31:H31"/>
+    <mergeCell ref="B86:B88"/>
+    <mergeCell ref="C74:C78"/>
+    <mergeCell ref="D74:D78"/>
+    <mergeCell ref="D79:D84"/>
+    <mergeCell ref="C79:C84"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C33:C36"/>
+    <mergeCell ref="D33:D36"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="D86:D88"/>
+    <mergeCell ref="C69:C73"/>
+    <mergeCell ref="C86:C88"/>
+    <mergeCell ref="E72:E73"/>
+    <mergeCell ref="B58:H58"/>
     <mergeCell ref="I15:I16"/>
     <mergeCell ref="I40:I41"/>
     <mergeCell ref="I61:I62"/>
@@ -4820,26 +4920,23 @@
     <mergeCell ref="D93:D96"/>
     <mergeCell ref="C93:C96"/>
     <mergeCell ref="I76:I77"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="C27:C29"/>
-    <mergeCell ref="D27:D29"/>
-    <mergeCell ref="B31:H31"/>
-    <mergeCell ref="B86:B88"/>
-    <mergeCell ref="C74:C78"/>
-    <mergeCell ref="D74:D78"/>
-    <mergeCell ref="D79:D84"/>
-    <mergeCell ref="C79:C84"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C33:C36"/>
-    <mergeCell ref="D33:D36"/>
-    <mergeCell ref="B33:B36"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="D86:D88"/>
-    <mergeCell ref="C69:C73"/>
-    <mergeCell ref="C86:C88"/>
-    <mergeCell ref="E72:E73"/>
-    <mergeCell ref="B58:H58"/>
+    <mergeCell ref="I106:I108"/>
+    <mergeCell ref="B118:B120"/>
+    <mergeCell ref="C118:C120"/>
+    <mergeCell ref="D118:D120"/>
+    <mergeCell ref="B109:H109"/>
+    <mergeCell ref="B44:H44"/>
+    <mergeCell ref="B49:H49"/>
+    <mergeCell ref="B53:H53"/>
+    <mergeCell ref="B106:B108"/>
+    <mergeCell ref="C106:C108"/>
+    <mergeCell ref="D106:D108"/>
+    <mergeCell ref="E106:E108"/>
+    <mergeCell ref="H106:H107"/>
+    <mergeCell ref="B64:H64"/>
+    <mergeCell ref="B85:H85"/>
+    <mergeCell ref="B74:B78"/>
+    <mergeCell ref="B79:B84"/>
     <mergeCell ref="B98:G98"/>
     <mergeCell ref="B104:B105"/>
     <mergeCell ref="E104:E105"/>
@@ -4847,66 +4944,6 @@
     <mergeCell ref="D89:D90"/>
     <mergeCell ref="C89:C90"/>
     <mergeCell ref="B97:H97"/>
-    <mergeCell ref="B89:B90"/>
-    <mergeCell ref="B93:B96"/>
-    <mergeCell ref="I104:I105"/>
-    <mergeCell ref="B99:B102"/>
-    <mergeCell ref="C99:C102"/>
-    <mergeCell ref="D99:D102"/>
-    <mergeCell ref="E101:E102"/>
-    <mergeCell ref="E99:E100"/>
-    <mergeCell ref="I99:I100"/>
-    <mergeCell ref="I101:I102"/>
-    <mergeCell ref="D104:D105"/>
-    <mergeCell ref="C104:C105"/>
-    <mergeCell ref="I86:I88"/>
-    <mergeCell ref="D69:D73"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="B9:B12"/>
-    <mergeCell ref="C9:C12"/>
-    <mergeCell ref="D9:D12"/>
-    <mergeCell ref="E9:E12"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="G9:G12"/>
-    <mergeCell ref="H9:H12"/>
-    <mergeCell ref="F9:F12"/>
-    <mergeCell ref="I9:I12"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="C19:C21"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="B117:I117"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="I38:I39"/>
-    <mergeCell ref="E76:E77"/>
-    <mergeCell ref="H65:H67"/>
-    <mergeCell ref="E70:E71"/>
-    <mergeCell ref="F46:F47"/>
-    <mergeCell ref="E28:E29"/>
-    <mergeCell ref="D19:D21"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="I65:I68"/>
-    <mergeCell ref="E79:E82"/>
-    <mergeCell ref="I79:I82"/>
-    <mergeCell ref="I19:I21"/>
-    <mergeCell ref="I22:I23"/>
-    <mergeCell ref="I28:I29"/>
-    <mergeCell ref="I34:I36"/>
-    <mergeCell ref="I70:I71"/>
-    <mergeCell ref="I72:I73"/>
-    <mergeCell ref="I74:I75"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>